<commit_message>
Integrate contract brief facts, Maximo validation, and corrections
Award $18.36M / 11.5 mi confirmed; $2M additive to $2.97M UG
credits. Corrections: sequencing ceiling ~$720-790k (15 CWOs =
~97% of OH program per Maximo); post-UG ~$1.34M/mi inside DTE's
own MPSC-audited range, $2M demand pushes below their floor;
PLS-verified $267k open commitments vs brief's $923k estimate.
Maximo validated against reconciliation (wire within 0.5%).
Scope-offset analyzed as solution and budget-vs-benchmark
diagnostic.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VrQFqy4MVniz1ZR4Ywwp9h
</commit_message>
<xml_diff>
--- a/new-baltimore/NBALT_Proto_Schedule_Sequencing_Model.xlsx
+++ b/new-baltimore/NBALT_Proto_Schedule_Sequencing_Model.xlsx
@@ -118,7 +118,7 @@
     <t xml:space="preserve">These 15 CWOs as share of total OH program</t>
   </si>
   <si>
-    <t xml:space="preserve">PLACEHOLDER — set from real program list (39 WOs incl. deleted UG)</t>
+    <t xml:space="preserve">REVISED from DTE Maximo workbook: our 15 CWOs cover ~97% of program install wire (141,020 ft total). Was 0.50 placeholder.</t>
   </si>
   <si>
     <t xml:space="preserve">CALENDAR</t>
@@ -1039,7 +1039,7 @@
         <v>30</v>
       </c>
       <c r="B20" s="10" t="n">
-        <v>0.5</v>
+        <v>0.95</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>31</v>
@@ -2343,15 +2343,15 @@
       </c>
       <c r="C17" s="23" t="n">
         <f aca="false">C16/Assumptions!$B$20</f>
-        <v>1364953.1656</v>
+        <v>718396.402947369</v>
       </c>
       <c r="D17" s="23" t="n">
         <f aca="false">D16/Assumptions!$B$20</f>
-        <v>1451040.6524</v>
+        <v>763705.606526316</v>
       </c>
       <c r="E17" s="23" t="n">
         <f aca="false">E16/Assumptions!$B$20</f>
-        <v>1494084.3958</v>
+        <v>786360.20831579</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>